<commit_message>
Update visa prediction model and application
</commit_message>
<xml_diff>
--- a/data_cleaned.xlsx
+++ b/data_cleaned.xlsx
@@ -949,7 +949,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Victorian Institute of Technology (VIT)</t>
+          <t xml:space="preserve">Victorian Institute of Technology (VIT) </t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Southern Academy of Business and Technology</t>
+          <t xml:space="preserve">Southern Academy of Business and Technology </t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -3950,7 +3950,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4416,7 +4416,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4475,7 +4475,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4650,7 +4650,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4884,7 +4884,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -5057,7 +5057,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -5114,7 +5114,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -5523,7 +5523,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -5639,7 +5639,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6331,7 +6331,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6390,7 +6390,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6565,7 +6565,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -6575,7 +6575,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6624,7 +6624,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6797,7 +6797,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t xml:space="preserve">Tidak </t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -7485,7 +7485,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -7495,7 +7495,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -7601,7 +7601,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Iya</t>
+          <t xml:space="preserve">Iya </t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>REFUSAL</t>
+          <t xml:space="preserve">REFUSAL </t>
         </is>
       </c>
     </row>

</xml_diff>